<commit_message>
SEND TO QC option in main_ui_themed
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/insights/image_folder_insight.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/insights/image_folder_insight.xlsx
@@ -43,7 +43,7 @@
       <color rgb="007A7A7A"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +75,11 @@
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,6 +125,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -575,8 +583,8 @@
       <c r="D2" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>1</v>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>2</v>
@@ -604,10 +612,10 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -616,10 +624,10 @@
         <v>0</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>0</v>
@@ -630,8 +638,8 @@
       <c r="J3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="4" t="n">
-        <v>12</v>
+      <c r="K3" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -647,7 +655,7 @@
         <v>9</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0</v>
@@ -752,34 +760,34 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="E7" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="K7" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -928,7 +936,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>20</v>
@@ -959,10 +967,10 @@
         <v>49</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>49</v>
@@ -971,10 +979,10 @@
         <v>49</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I3" s="4" t="n">
         <v>49</v>
@@ -986,7 +994,7 @@
         <v>49</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -1005,7 +1013,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>29</v>
@@ -1119,22 +1127,22 @@
         <v>81</v>
       </c>
       <c r="C7" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>64</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>51</v>
-      </c>
       <c r="F7" s="4" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>81</v>
@@ -1143,10 +1151,10 @@
         <v>81</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8">
@@ -1200,10 +1208,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1291,6 +1299,48 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Warnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Ice: skipped folder tokens in '1-FADE'f-FADE's-IND'f-STAR'f-STAR's - Aps' (Unknown brand code 'Aps' in folder '1-FADE'f-FADE's-IND'f-STAR'f-STAR's - Aps')</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Ice: skipped folder tokens in '2-FADE'f-FADE's-IND'f-STAR'f-STAR's - As' (Unknown brand code 'As' in folder '2-FADE'f-FADE's-IND'f-STAR'f-STAR's - As')</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ice: skipped folder tokens in '3-FADE'f-FADE's-IND'f-STAR'f-STAR's - As' (Unknown brand code 'As' in folder '3-FADE'f-FADE's-IND'f-STAR'f-STAR's - As')</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Trouser: skipped folder tokens in '1-FADE'f-FADE's-GENZ'f-GENZ's-IND'f-IND's-STAR'f-STAR's - Aps' (Unknown brand code 'Aps' in folder '1-FADE'f-FADE's-GENZ'f-GENZ's-IND'f-IND's-STAR'f-STAR's - Aps')</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Trouser: skipped folder tokens in '2-FADE'f-FADE's-GENZ'f-GENZ's-IND'f-IND's-STAR'f-STAR's -Aps' (Unknown brand code 'Aps' in folder '2-FADE'f-FADE's-GENZ'f-GENZ's-IND'f-IND's-STAR'f-STAR's -Aps')</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>